<commit_message>
Two-country hub layout; add US atlas
</commit_message>
<xml_diff>
--- a/UK_Model_Archive.xlsx
+++ b/UK_Model_Archive.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2990,6 +2990,454 @@
       </c>
       <c r="H91" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>19</v>
+      </c>
+      <c r="C92" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D92" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E92" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F92" t="n">
+        <v>3</v>
+      </c>
+      <c r="G92" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>19</v>
+      </c>
+      <c r="C93" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D93" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E93" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F93" t="n">
+        <v>3</v>
+      </c>
+      <c r="G93" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>19</v>
+      </c>
+      <c r="C94" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D94" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E94" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F94" t="n">
+        <v>3</v>
+      </c>
+      <c r="G94" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>19</v>
+      </c>
+      <c r="C95" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D95" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E95" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F95" t="n">
+        <v>3</v>
+      </c>
+      <c r="G95" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>19</v>
+      </c>
+      <c r="C96" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D96" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E96" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F96" t="n">
+        <v>3</v>
+      </c>
+      <c r="G96" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>19</v>
+      </c>
+      <c r="C97" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D97" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E97" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F97" t="n">
+        <v>3</v>
+      </c>
+      <c r="G97" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>19</v>
+      </c>
+      <c r="C98" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="D98" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E98" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="F98" t="n">
+        <v>3</v>
+      </c>
+      <c r="G98" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="H98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C99" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D99" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E99" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F99" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G99" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C100" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D100" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E100" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F100" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G100" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C101" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D101" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E101" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F101" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G101" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C102" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D102" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E102" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F102" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G102" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C103" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D103" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E103" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F103" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G103" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C104" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D104" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E104" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F104" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G104" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C105" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D105" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E105" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F105" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G105" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>18.55056247991314</v>
+      </c>
+      <c r="C106" t="n">
+        <v>17.95204089413426</v>
+      </c>
+      <c r="D106" t="n">
+        <v>12.70947221310472</v>
+      </c>
+      <c r="E106" t="n">
+        <v>14.30048663675842</v>
+      </c>
+      <c r="F106" t="n">
+        <v>3.50219300119863</v>
+      </c>
+      <c r="G106" t="n">
+        <v>27.43251275103527</v>
+      </c>
+      <c r="H106" t="n">
+        <v>0.9000010133445013</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>18.54639458566736</v>
+      </c>
+      <c r="C107" t="n">
+        <v>18.05862601916582</v>
+      </c>
+      <c r="D107" t="n">
+        <v>12.35197449779278</v>
+      </c>
+      <c r="E107" t="n">
+        <v>14.97082258365463</v>
+      </c>
+      <c r="F107" t="n">
+        <v>3.265001686209501</v>
+      </c>
+      <c r="G107" t="n">
+        <v>27.24872948241329</v>
+      </c>
+      <c r="H107" t="n">
+        <v>1.135047504724195</v>
       </c>
     </row>
   </sheetData>
@@ -3003,7 +3451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7216,6 +7664,742 @@
       </c>
       <c r="N91" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>126</v>
+      </c>
+      <c r="C92" t="n">
+        <v>83</v>
+      </c>
+      <c r="D92" t="n">
+        <v>71</v>
+      </c>
+      <c r="E92" t="n">
+        <v>10</v>
+      </c>
+      <c r="F92" t="n">
+        <v>47</v>
+      </c>
+      <c r="G92" t="n">
+        <v>280</v>
+      </c>
+      <c r="H92" t="n">
+        <v>6</v>
+      </c>
+      <c r="I92" t="n">
+        <v>1</v>
+      </c>
+      <c r="J92" t="n">
+        <v>10</v>
+      </c>
+      <c r="K92" t="n">
+        <v>2</v>
+      </c>
+      <c r="L92" t="n">
+        <v>2</v>
+      </c>
+      <c r="M92" t="n">
+        <v>1</v>
+      </c>
+      <c r="N92" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>123</v>
+      </c>
+      <c r="C93" t="n">
+        <v>83</v>
+      </c>
+      <c r="D93" t="n">
+        <v>71</v>
+      </c>
+      <c r="E93" t="n">
+        <v>10</v>
+      </c>
+      <c r="F93" t="n">
+        <v>47</v>
+      </c>
+      <c r="G93" t="n">
+        <v>283</v>
+      </c>
+      <c r="H93" t="n">
+        <v>6</v>
+      </c>
+      <c r="I93" t="n">
+        <v>1</v>
+      </c>
+      <c r="J93" t="n">
+        <v>10</v>
+      </c>
+      <c r="K93" t="n">
+        <v>2</v>
+      </c>
+      <c r="L93" t="n">
+        <v>2</v>
+      </c>
+      <c r="M93" t="n">
+        <v>1</v>
+      </c>
+      <c r="N93" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>126</v>
+      </c>
+      <c r="C94" t="n">
+        <v>84</v>
+      </c>
+      <c r="D94" t="n">
+        <v>71</v>
+      </c>
+      <c r="E94" t="n">
+        <v>10</v>
+      </c>
+      <c r="F94" t="n">
+        <v>47</v>
+      </c>
+      <c r="G94" t="n">
+        <v>279</v>
+      </c>
+      <c r="H94" t="n">
+        <v>6</v>
+      </c>
+      <c r="I94" t="n">
+        <v>1</v>
+      </c>
+      <c r="J94" t="n">
+        <v>10</v>
+      </c>
+      <c r="K94" t="n">
+        <v>2</v>
+      </c>
+      <c r="L94" t="n">
+        <v>2</v>
+      </c>
+      <c r="M94" t="n">
+        <v>1</v>
+      </c>
+      <c r="N94" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>125</v>
+      </c>
+      <c r="C95" t="n">
+        <v>83</v>
+      </c>
+      <c r="D95" t="n">
+        <v>71</v>
+      </c>
+      <c r="E95" t="n">
+        <v>10</v>
+      </c>
+      <c r="F95" t="n">
+        <v>47</v>
+      </c>
+      <c r="G95" t="n">
+        <v>281</v>
+      </c>
+      <c r="H95" t="n">
+        <v>6</v>
+      </c>
+      <c r="I95" t="n">
+        <v>1</v>
+      </c>
+      <c r="J95" t="n">
+        <v>10</v>
+      </c>
+      <c r="K95" t="n">
+        <v>2</v>
+      </c>
+      <c r="L95" t="n">
+        <v>2</v>
+      </c>
+      <c r="M95" t="n">
+        <v>1</v>
+      </c>
+      <c r="N95" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>124</v>
+      </c>
+      <c r="C96" t="n">
+        <v>83</v>
+      </c>
+      <c r="D96" t="n">
+        <v>71</v>
+      </c>
+      <c r="E96" t="n">
+        <v>10</v>
+      </c>
+      <c r="F96" t="n">
+        <v>47</v>
+      </c>
+      <c r="G96" t="n">
+        <v>282</v>
+      </c>
+      <c r="H96" t="n">
+        <v>6</v>
+      </c>
+      <c r="I96" t="n">
+        <v>1</v>
+      </c>
+      <c r="J96" t="n">
+        <v>10</v>
+      </c>
+      <c r="K96" t="n">
+        <v>2</v>
+      </c>
+      <c r="L96" t="n">
+        <v>2</v>
+      </c>
+      <c r="M96" t="n">
+        <v>1</v>
+      </c>
+      <c r="N96" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>123</v>
+      </c>
+      <c r="C97" t="n">
+        <v>83</v>
+      </c>
+      <c r="D97" t="n">
+        <v>71</v>
+      </c>
+      <c r="E97" t="n">
+        <v>10</v>
+      </c>
+      <c r="F97" t="n">
+        <v>47</v>
+      </c>
+      <c r="G97" t="n">
+        <v>283</v>
+      </c>
+      <c r="H97" t="n">
+        <v>6</v>
+      </c>
+      <c r="I97" t="n">
+        <v>1</v>
+      </c>
+      <c r="J97" t="n">
+        <v>10</v>
+      </c>
+      <c r="K97" t="n">
+        <v>2</v>
+      </c>
+      <c r="L97" t="n">
+        <v>2</v>
+      </c>
+      <c r="M97" t="n">
+        <v>1</v>
+      </c>
+      <c r="N97" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>125</v>
+      </c>
+      <c r="C98" t="n">
+        <v>84</v>
+      </c>
+      <c r="D98" t="n">
+        <v>71</v>
+      </c>
+      <c r="E98" t="n">
+        <v>10</v>
+      </c>
+      <c r="F98" t="n">
+        <v>47</v>
+      </c>
+      <c r="G98" t="n">
+        <v>280</v>
+      </c>
+      <c r="H98" t="n">
+        <v>6</v>
+      </c>
+      <c r="I98" t="n">
+        <v>1</v>
+      </c>
+      <c r="J98" t="n">
+        <v>10</v>
+      </c>
+      <c r="K98" t="n">
+        <v>2</v>
+      </c>
+      <c r="L98" t="n">
+        <v>2</v>
+      </c>
+      <c r="M98" t="n">
+        <v>1</v>
+      </c>
+      <c r="N98" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="n">
+        <v>632</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>6</v>
+      </c>
+      <c r="K99" t="n">
+        <v>2</v>
+      </c>
+      <c r="L99" t="n">
+        <v>7</v>
+      </c>
+      <c r="M99" t="n">
+        <v>1</v>
+      </c>
+      <c r="N99" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>159</v>
+      </c>
+      <c r="C100" t="n">
+        <v>77</v>
+      </c>
+      <c r="D100" t="n">
+        <v>83</v>
+      </c>
+      <c r="E100" t="n">
+        <v>12</v>
+      </c>
+      <c r="F100" t="n">
+        <v>26</v>
+      </c>
+      <c r="G100" t="n">
+        <v>256</v>
+      </c>
+      <c r="H100" t="n">
+        <v>4</v>
+      </c>
+      <c r="I100" t="n">
+        <v>15</v>
+      </c>
+      <c r="J100" t="n">
+        <v>6</v>
+      </c>
+      <c r="K100" t="n">
+        <v>2</v>
+      </c>
+      <c r="L100" t="n">
+        <v>7</v>
+      </c>
+      <c r="M100" t="n">
+        <v>1</v>
+      </c>
+      <c r="N100" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>158</v>
+      </c>
+      <c r="C101" t="n">
+        <v>78</v>
+      </c>
+      <c r="D101" t="n">
+        <v>83</v>
+      </c>
+      <c r="E101" t="n">
+        <v>12</v>
+      </c>
+      <c r="F101" t="n">
+        <v>26</v>
+      </c>
+      <c r="G101" t="n">
+        <v>254</v>
+      </c>
+      <c r="H101" t="n">
+        <v>4</v>
+      </c>
+      <c r="I101" t="n">
+        <v>17</v>
+      </c>
+      <c r="J101" t="n">
+        <v>6</v>
+      </c>
+      <c r="K101" t="n">
+        <v>2</v>
+      </c>
+      <c r="L101" t="n">
+        <v>7</v>
+      </c>
+      <c r="M101" t="n">
+        <v>1</v>
+      </c>
+      <c r="N101" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>159</v>
+      </c>
+      <c r="C102" t="n">
+        <v>81</v>
+      </c>
+      <c r="D102" t="n">
+        <v>80</v>
+      </c>
+      <c r="E102" t="n">
+        <v>7</v>
+      </c>
+      <c r="F102" t="n">
+        <v>27</v>
+      </c>
+      <c r="G102" t="n">
+        <v>259</v>
+      </c>
+      <c r="H102" t="n">
+        <v>4</v>
+      </c>
+      <c r="I102" t="n">
+        <v>15</v>
+      </c>
+      <c r="J102" t="n">
+        <v>6</v>
+      </c>
+      <c r="K102" t="n">
+        <v>2</v>
+      </c>
+      <c r="L102" t="n">
+        <v>7</v>
+      </c>
+      <c r="M102" t="n">
+        <v>1</v>
+      </c>
+      <c r="N102" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>159</v>
+      </c>
+      <c r="C103" t="n">
+        <v>83</v>
+      </c>
+      <c r="D103" t="n">
+        <v>80</v>
+      </c>
+      <c r="E103" t="n">
+        <v>7</v>
+      </c>
+      <c r="F103" t="n">
+        <v>27</v>
+      </c>
+      <c r="G103" t="n">
+        <v>257</v>
+      </c>
+      <c r="H103" t="n">
+        <v>4</v>
+      </c>
+      <c r="I103" t="n">
+        <v>15</v>
+      </c>
+      <c r="J103" t="n">
+        <v>6</v>
+      </c>
+      <c r="K103" t="n">
+        <v>2</v>
+      </c>
+      <c r="L103" t="n">
+        <v>7</v>
+      </c>
+      <c r="M103" t="n">
+        <v>1</v>
+      </c>
+      <c r="N103" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>159</v>
+      </c>
+      <c r="C104" t="n">
+        <v>80</v>
+      </c>
+      <c r="D104" t="n">
+        <v>80</v>
+      </c>
+      <c r="E104" t="n">
+        <v>7</v>
+      </c>
+      <c r="F104" t="n">
+        <v>27</v>
+      </c>
+      <c r="G104" t="n">
+        <v>260</v>
+      </c>
+      <c r="H104" t="n">
+        <v>4</v>
+      </c>
+      <c r="I104" t="n">
+        <v>15</v>
+      </c>
+      <c r="J104" t="n">
+        <v>6</v>
+      </c>
+      <c r="K104" t="n">
+        <v>2</v>
+      </c>
+      <c r="L104" t="n">
+        <v>7</v>
+      </c>
+      <c r="M104" t="n">
+        <v>1</v>
+      </c>
+      <c r="N104" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>160</v>
+      </c>
+      <c r="C105" t="n">
+        <v>69</v>
+      </c>
+      <c r="D105" t="n">
+        <v>80</v>
+      </c>
+      <c r="E105" t="n">
+        <v>8</v>
+      </c>
+      <c r="F105" t="n">
+        <v>26</v>
+      </c>
+      <c r="G105" t="n">
+        <v>270</v>
+      </c>
+      <c r="H105" t="n">
+        <v>4</v>
+      </c>
+      <c r="I105" t="n">
+        <v>15</v>
+      </c>
+      <c r="J105" t="n">
+        <v>6</v>
+      </c>
+      <c r="K105" t="n">
+        <v>2</v>
+      </c>
+      <c r="L105" t="n">
+        <v>7</v>
+      </c>
+      <c r="M105" t="n">
+        <v>1</v>
+      </c>
+      <c r="N105" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>161</v>
+      </c>
+      <c r="C106" t="n">
+        <v>69</v>
+      </c>
+      <c r="D106" t="n">
+        <v>80</v>
+      </c>
+      <c r="E106" t="n">
+        <v>8</v>
+      </c>
+      <c r="F106" t="n">
+        <v>26</v>
+      </c>
+      <c r="G106" t="n">
+        <v>269</v>
+      </c>
+      <c r="H106" t="n">
+        <v>4</v>
+      </c>
+      <c r="I106" t="n">
+        <v>15</v>
+      </c>
+      <c r="J106" t="n">
+        <v>6</v>
+      </c>
+      <c r="K106" t="n">
+        <v>2</v>
+      </c>
+      <c r="L106" t="n">
+        <v>7</v>
+      </c>
+      <c r="M106" t="n">
+        <v>1</v>
+      </c>
+      <c r="N106" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>145</v>
+      </c>
+      <c r="C107" t="n">
+        <v>74</v>
+      </c>
+      <c r="D107" t="n">
+        <v>78</v>
+      </c>
+      <c r="E107" t="n">
+        <v>14</v>
+      </c>
+      <c r="F107" t="n">
+        <v>26</v>
+      </c>
+      <c r="G107" t="n">
+        <v>277</v>
+      </c>
+      <c r="H107" t="n">
+        <v>4</v>
+      </c>
+      <c r="I107" t="n">
+        <v>14</v>
+      </c>
+      <c r="J107" t="n">
+        <v>6</v>
+      </c>
+      <c r="K107" t="n">
+        <v>2</v>
+      </c>
+      <c r="L107" t="n">
+        <v>7</v>
+      </c>
+      <c r="M107" t="n">
+        <v>1</v>
+      </c>
+      <c r="N107" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -7229,7 +8413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7263,6 +8447,16 @@
           <t>Other</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LD_Maj</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>REF_Maj</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7285,6 +8479,8 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7307,6 +8503,8 @@
       <c r="F3" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7329,6 +8527,8 @@
       <c r="F4" t="n">
         <v>0</v>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7351,6 +8551,8 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7373,6 +8575,8 @@
       <c r="F6" t="n">
         <v>0</v>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7395,6 +8599,8 @@
       <c r="F7" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7417,6 +8623,8 @@
       <c r="F8" t="n">
         <v>0</v>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7439,6 +8647,8 @@
       <c r="F9" t="n">
         <v>0</v>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7461,6 +8671,8 @@
       <c r="F10" t="n">
         <v>0</v>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7483,6 +8695,8 @@
       <c r="F11" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7505,6 +8719,8 @@
       <c r="F12" t="n">
         <v>0</v>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7527,6 +8743,8 @@
       <c r="F13" t="n">
         <v>0</v>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7549,6 +8767,8 @@
       <c r="F14" t="n">
         <v>0.1000000000000085</v>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7571,6 +8791,8 @@
       <c r="F15" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7593,6 +8815,8 @@
       <c r="F16" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7615,6 +8839,8 @@
       <c r="F17" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7637,6 +8863,8 @@
       <c r="F18" t="n">
         <v>-0.1000000000000085</v>
       </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7659,6 +8887,8 @@
       <c r="F19" t="n">
         <v>0</v>
       </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7681,6 +8911,8 @@
       <c r="F20" t="n">
         <v>1.4210854715202e-14</v>
       </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7703,6 +8935,8 @@
       <c r="F21" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7725,6 +8959,8 @@
       <c r="F22" t="n">
         <v>0</v>
       </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7747,6 +8983,8 @@
       <c r="F23" t="n">
         <v>0</v>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7769,6 +9007,8 @@
       <c r="F24" t="n">
         <v>0</v>
       </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7791,6 +9031,8 @@
       <c r="F25" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7813,6 +9055,8 @@
       <c r="F26" t="n">
         <v>0</v>
       </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7835,6 +9079,8 @@
       <c r="F27" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7857,6 +9103,8 @@
       <c r="F28" t="n">
         <v>0</v>
       </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7879,6 +9127,8 @@
       <c r="F29" t="n">
         <v>0</v>
       </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7901,6 +9151,8 @@
       <c r="F30" t="n">
         <v>0</v>
       </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7923,6 +9175,8 @@
       <c r="F31" t="n">
         <v>0</v>
       </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7945,6 +9199,8 @@
       <c r="F32" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7967,6 +9223,8 @@
       <c r="F33" t="n">
         <v>0</v>
       </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7989,6 +9247,8 @@
       <c r="F34" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8011,6 +9271,8 @@
       <c r="F35" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8033,6 +9295,8 @@
       <c r="F36" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8055,6 +9319,8 @@
       <c r="F37" t="n">
         <v>-0.1000000000000085</v>
       </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8077,6 +9343,8 @@
       <c r="F38" t="n">
         <v>0</v>
       </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8099,6 +9367,8 @@
       <c r="F39" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8121,6 +9391,8 @@
       <c r="F40" t="n">
         <v>0</v>
       </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8143,6 +9415,8 @@
       <c r="F41" t="n">
         <v>0</v>
       </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8165,6 +9439,8 @@
       <c r="F42" t="n">
         <v>0</v>
       </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8187,6 +9463,8 @@
       <c r="F43" t="n">
         <v>0</v>
       </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8209,6 +9487,8 @@
       <c r="F44" t="n">
         <v>0</v>
       </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8231,6 +9511,8 @@
       <c r="F45" t="n">
         <v>0</v>
       </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8253,6 +9535,8 @@
       <c r="F46" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8275,6 +9559,8 @@
       <c r="F47" t="n">
         <v>0</v>
       </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8297,6 +9583,8 @@
       <c r="F48" t="n">
         <v>0</v>
       </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8319,6 +9607,8 @@
       <c r="F49" t="n">
         <v>0</v>
       </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8341,6 +9631,8 @@
       <c r="F50" t="n">
         <v>0</v>
       </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8363,6 +9655,8 @@
       <c r="F51" t="n">
         <v>0</v>
       </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8385,6 +9679,8 @@
       <c r="F52" t="n">
         <v>0.1000000000000085</v>
       </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8407,6 +9703,8 @@
       <c r="F53" t="n">
         <v>0</v>
       </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8429,6 +9727,8 @@
       <c r="F54" t="n">
         <v>0</v>
       </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8451,6 +9751,8 @@
       <c r="F55" t="n">
         <v>1.4210854715202e-14</v>
       </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8473,6 +9775,8 @@
       <c r="F56" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8495,6 +9799,8 @@
       <c r="F57" t="n">
         <v>0</v>
       </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8517,6 +9823,8 @@
       <c r="F58" t="n">
         <v>0</v>
       </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8539,6 +9847,8 @@
       <c r="F59" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8561,6 +9871,8 @@
       <c r="F60" t="n">
         <v>0</v>
       </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8583,6 +9895,8 @@
       <c r="F61" t="n">
         <v>1.4210854715202e-14</v>
       </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8605,6 +9919,8 @@
       <c r="F62" t="n">
         <v>0</v>
       </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8627,6 +9943,8 @@
       <c r="F63" t="n">
         <v>0</v>
       </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8649,6 +9967,8 @@
       <c r="F64" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8671,6 +9991,8 @@
       <c r="F65" t="n">
         <v>0</v>
       </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8693,6 +10015,8 @@
       <c r="F66" t="n">
         <v>0</v>
       </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8715,6 +10039,8 @@
       <c r="F67" t="n">
         <v>1.4210854715202e-14</v>
       </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8737,6 +10063,8 @@
       <c r="F68" t="n">
         <v>0</v>
       </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8759,6 +10087,8 @@
       <c r="F69" t="n">
         <v>0</v>
       </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8781,6 +10111,8 @@
       <c r="F70" t="n">
         <v>0</v>
       </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8803,6 +10135,8 @@
       <c r="F71" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8825,6 +10159,8 @@
       <c r="F72" t="n">
         <v>0</v>
       </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8847,6 +10183,8 @@
       <c r="F73" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8869,6 +10207,8 @@
       <c r="F74" t="n">
         <v>0.1000000000000085</v>
       </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8891,6 +10231,8 @@
       <c r="F75" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8913,6 +10255,8 @@
       <c r="F76" t="n">
         <v>0.1000000000000085</v>
       </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8935,6 +10279,8 @@
       <c r="F77" t="n">
         <v>-1.4210854715202e-14</v>
       </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8957,6 +10303,8 @@
       <c r="F78" t="n">
         <v>0</v>
       </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8979,6 +10327,8 @@
       <c r="F79" t="n">
         <v>0</v>
       </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9001,6 +10351,8 @@
       <c r="F80" t="n">
         <v>0</v>
       </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9023,6 +10375,8 @@
       <c r="F81" t="n">
         <v>-0.09999999999999432</v>
       </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9045,6 +10399,8 @@
       <c r="F82" t="n">
         <v>0</v>
       </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9067,6 +10423,8 @@
       <c r="F83" t="n">
         <v>0</v>
       </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9089,6 +10447,8 @@
       <c r="F84" t="n">
         <v>1.4210854715202e-14</v>
       </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9111,6 +10471,8 @@
       <c r="F85" t="n">
         <v>0.09999999999999432</v>
       </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9133,6 +10495,8 @@
       <c r="F86" t="n">
         <v>0.5999999999999943</v>
       </c>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9155,6 +10519,8 @@
       <c r="F87" t="n">
         <v>86</v>
       </c>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9177,6 +10543,8 @@
       <c r="F88" t="n">
         <v>86.5</v>
       </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9199,6 +10567,8 @@
       <c r="F89" t="n">
         <v>94.59999999999999</v>
       </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9221,6 +10591,8 @@
       <c r="F90" t="n">
         <v>94.5</v>
       </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9242,6 +10614,428 @@
       </c>
       <c r="F91" t="n">
         <v>94.5</v>
+      </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F92" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F94" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F96" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D97" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F97" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="n">
+        <v>3</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F98" t="n">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" t="n">
+        <v>100</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C100" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F100" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="n">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C101" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F101" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C102" t="n">
+        <v>18</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F102" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C103" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F103" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C104" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F104" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="n">
+        <v>17.9</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C105" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F105" t="n">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="n">
+        <v>17.8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C106" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="D106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F106" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C107" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="n">
+        <v>21.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>